<commit_message>
feat: release v0.9.0 ledger writeback
</commit_message>
<xml_diff>
--- a/src/purchase_tool/web/买家号统一台账模板.xlsx
+++ b/src/purchase_tool/web/买家号统一台账模板.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="买家号统一台账" sheetId="1" r:id="Rfeead69647364c67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段配置说明" sheetId="2" r:id="Re46768acf7734730"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="买家号统一台账" sheetId="1" r:id="Re1bf5b1718024c54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段配置说明" sheetId="2" r:id="Rab035b3fdd0f492a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -85,7 +85,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -147,8 +147,13 @@
         <x:fgColor rgb="FFF2F5F8"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F2742"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="6">
+  <x:borders count="7">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -193,11 +198,25 @@
         <x:color rgb="FFD9E2EA"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF0F2742"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF0F2742"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF0F2742"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF0F2742"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="120">
+  <x:cellXfs count="125">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -436,6 +455,15 @@
     <x:xf numFmtId="0" fontId="9" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -458,7 +486,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -672,18 +700,19 @@
     <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="13" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="24" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="19" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="19" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="17" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="19" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="17" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="17" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="28" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="14" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="28" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="18" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="22" hidden="0" customWidth="1"/>
-    <x:col min="22" max="22" width="18" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="17" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="28" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="14" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="28" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="18" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="22" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -718,39 +747,42 @@
         <x:v>绑定环境</x:v>
       </x:c>
       <x:c r="K1" s="77" t="str">
+        <x:v>环境分组名</x:v>
+      </x:c>
+      <x:c r="L1" s="77" t="str">
         <x:v>环境序号</x:v>
       </x:c>
-      <x:c r="L1" s="77" t="str">
+      <x:c r="M1" s="77" t="str">
         <x:v>采购员</x:v>
       </x:c>
-      <x:c r="M1" s="77" t="str">
+      <x:c r="N1" s="77" t="str">
         <x:v>绑定时间</x:v>
       </x:c>
-      <x:c r="N1" s="77" t="str">
+      <x:c r="O1" s="77" t="str">
         <x:v>首次登录日期</x:v>
       </x:c>
-      <x:c r="O1" s="77" t="str">
+      <x:c r="P1" s="77" t="str">
         <x:v>最后使用日期</x:v>
       </x:c>
-      <x:c r="P1" s="77" t="str">
+      <x:c r="Q1" s="77" t="str">
         <x:v>创建时间</x:v>
       </x:c>
-      <x:c r="Q1" s="77" t="str">
+      <x:c r="R1" s="77" t="str">
         <x:v>备注</x:v>
       </x:c>
-      <x:c r="R1" s="77" t="str">
+      <x:c r="S1" s="77" t="str">
         <x:v>累计下单数</x:v>
       </x:c>
-      <x:c r="S1" s="77" t="str">
+      <x:c r="T1" s="77" t="str">
         <x:v>异常记录</x:v>
       </x:c>
-      <x:c r="T1" s="77" t="str">
+      <x:c r="U1" s="77" t="str">
         <x:v>创建人</x:v>
       </x:c>
-      <x:c r="U1" s="77" t="str">
+      <x:c r="V1" s="78" t="str">
         <x:v>迁移状态</x:v>
       </x:c>
-      <x:c r="V1" s="78" t="str">
+      <x:c r="W1" s="124" t="str">
         <x:v>操作人</x:v>
       </x:c>
     </x:row>
@@ -777,6 +809,7 @@
       <x:c r="T2" s="83"/>
       <x:c r="U2" s="83"/>
       <x:c r="V2" s="83"/>
+      <x:c r="W2"/>
     </x:row>
     <x:row r="3" ht="23" customHeight="1">
       <x:c r="A3" s="84"/>
@@ -801,6 +834,7 @@
       <x:c r="T3" s="84"/>
       <x:c r="U3" s="84"/>
       <x:c r="V3" s="84"/>
+      <x:c r="W3"/>
     </x:row>
     <x:row r="4" ht="23" customHeight="1">
       <x:c r="A4" s="84"/>
@@ -825,6 +859,7 @@
       <x:c r="T4" s="84"/>
       <x:c r="U4" s="84"/>
       <x:c r="V4" s="84"/>
+      <x:c r="W4"/>
     </x:row>
     <x:row r="5" ht="23" customHeight="1">
       <x:c r="A5" s="84"/>
@@ -849,6 +884,7 @@
       <x:c r="T5" s="84"/>
       <x:c r="U5" s="84"/>
       <x:c r="V5" s="84"/>
+      <x:c r="W5"/>
     </x:row>
     <x:row r="6" ht="23" customHeight="1">
       <x:c r="A6" s="84"/>
@@ -873,6 +909,7 @@
       <x:c r="T6" s="84"/>
       <x:c r="U6" s="84"/>
       <x:c r="V6" s="84"/>
+      <x:c r="W6"/>
     </x:row>
     <x:row r="7" ht="23" customHeight="1">
       <x:c r="A7" s="84"/>
@@ -897,6 +934,7 @@
       <x:c r="T7" s="84"/>
       <x:c r="U7" s="84"/>
       <x:c r="V7" s="84"/>
+      <x:c r="W7"/>
     </x:row>
     <x:row r="8" ht="23" customHeight="1">
       <x:c r="A8" s="84"/>
@@ -921,6 +959,7 @@
       <x:c r="T8" s="84"/>
       <x:c r="U8" s="84"/>
       <x:c r="V8" s="84"/>
+      <x:c r="W8"/>
     </x:row>
     <x:row r="9" ht="23" customHeight="1">
       <x:c r="A9" s="84"/>
@@ -945,6 +984,7 @@
       <x:c r="T9" s="84"/>
       <x:c r="U9" s="84"/>
       <x:c r="V9" s="84"/>
+      <x:c r="W9"/>
     </x:row>
     <x:row r="10" ht="23" customHeight="1">
       <x:c r="A10" s="84"/>
@@ -969,6 +1009,7 @@
       <x:c r="T10" s="84"/>
       <x:c r="U10" s="84"/>
       <x:c r="V10" s="84"/>
+      <x:c r="W10"/>
     </x:row>
     <x:row r="11" ht="23" customHeight="1">
       <x:c r="A11" s="84"/>
@@ -993,6 +1034,7 @@
       <x:c r="T11" s="84"/>
       <x:c r="U11" s="84"/>
       <x:c r="V11" s="84"/>
+      <x:c r="W11"/>
     </x:row>
     <x:row r="12" ht="23" customHeight="1">
       <x:c r="A12" s="84"/>
@@ -1017,6 +1059,7 @@
       <x:c r="T12" s="84"/>
       <x:c r="U12" s="84"/>
       <x:c r="V12" s="84"/>
+      <x:c r="W12"/>
     </x:row>
     <x:row r="13" ht="23" customHeight="1">
       <x:c r="A13" s="84"/>
@@ -1041,6 +1084,7 @@
       <x:c r="T13" s="84"/>
       <x:c r="U13" s="84"/>
       <x:c r="V13" s="84"/>
+      <x:c r="W13"/>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">
       <x:c r="A14" s="84"/>
@@ -1065,6 +1109,7 @@
       <x:c r="T14" s="84"/>
       <x:c r="U14" s="84"/>
       <x:c r="V14" s="84"/>
+      <x:c r="W14"/>
     </x:row>
     <x:row r="15" ht="23" customHeight="1">
       <x:c r="A15" s="84"/>
@@ -1089,6 +1134,7 @@
       <x:c r="T15" s="84"/>
       <x:c r="U15" s="84"/>
       <x:c r="V15" s="84"/>
+      <x:c r="W15"/>
     </x:row>
     <x:row r="16" ht="23" customHeight="1">
       <x:c r="A16" s="84"/>
@@ -1113,6 +1159,7 @@
       <x:c r="T16" s="84"/>
       <x:c r="U16" s="84"/>
       <x:c r="V16" s="84"/>
+      <x:c r="W16"/>
     </x:row>
     <x:row r="17" ht="23" customHeight="1">
       <x:c r="A17" s="84"/>
@@ -1137,6 +1184,7 @@
       <x:c r="T17" s="84"/>
       <x:c r="U17" s="84"/>
       <x:c r="V17" s="84"/>
+      <x:c r="W17"/>
     </x:row>
     <x:row r="18" ht="23" customHeight="1">
       <x:c r="A18" s="84"/>
@@ -1161,6 +1209,7 @@
       <x:c r="T18" s="84"/>
       <x:c r="U18" s="84"/>
       <x:c r="V18" s="84"/>
+      <x:c r="W18"/>
     </x:row>
     <x:row r="19" ht="23" customHeight="1">
       <x:c r="A19" s="84"/>
@@ -1185,6 +1234,7 @@
       <x:c r="T19" s="84"/>
       <x:c r="U19" s="84"/>
       <x:c r="V19" s="84"/>
+      <x:c r="W19"/>
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
       <x:c r="A20" s="84"/>
@@ -1209,6 +1259,7 @@
       <x:c r="T20" s="84"/>
       <x:c r="U20" s="84"/>
       <x:c r="V20" s="84"/>
+      <x:c r="W20"/>
     </x:row>
     <x:row r="21" ht="23" customHeight="1">
       <x:c r="A21" s="84"/>
@@ -1233,6 +1284,7 @@
       <x:c r="T21" s="84"/>
       <x:c r="U21" s="84"/>
       <x:c r="V21" s="84"/>
+      <x:c r="W21"/>
     </x:row>
     <x:row r="22" ht="23" customHeight="1">
       <x:c r="A22" s="84"/>
@@ -1257,6 +1309,7 @@
       <x:c r="T22" s="84"/>
       <x:c r="U22" s="84"/>
       <x:c r="V22" s="84"/>
+      <x:c r="W22"/>
     </x:row>
     <x:row r="23" ht="23" customHeight="1">
       <x:c r="A23" s="84"/>
@@ -1281,6 +1334,7 @@
       <x:c r="T23" s="84"/>
       <x:c r="U23" s="84"/>
       <x:c r="V23" s="84"/>
+      <x:c r="W23"/>
     </x:row>
     <x:row r="24" ht="23" customHeight="1">
       <x:c r="A24" s="84"/>
@@ -1305,6 +1359,7 @@
       <x:c r="T24" s="84"/>
       <x:c r="U24" s="84"/>
       <x:c r="V24" s="84"/>
+      <x:c r="W24"/>
     </x:row>
     <x:row r="25" ht="23" customHeight="1">
       <x:c r="A25" s="84"/>
@@ -1329,6 +1384,7 @@
       <x:c r="T25" s="84"/>
       <x:c r="U25" s="84"/>
       <x:c r="V25" s="84"/>
+      <x:c r="W25"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="21"/>
@@ -1353,6 +1409,7 @@
       <x:c r="T26" s="21"/>
       <x:c r="U26" s="21"/>
       <x:c r="V26" s="21"/>
+      <x:c r="W26"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="21"/>
@@ -1377,6 +1434,7 @@
       <x:c r="T27" s="21"/>
       <x:c r="U27" s="21"/>
       <x:c r="V27" s="21"/>
+      <x:c r="W27"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="21"/>
@@ -1401,6 +1459,7 @@
       <x:c r="T28" s="21"/>
       <x:c r="U28" s="21"/>
       <x:c r="V28" s="21"/>
+      <x:c r="W28"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="21"/>
@@ -1425,6 +1484,7 @@
       <x:c r="T29" s="21"/>
       <x:c r="U29" s="21"/>
       <x:c r="V29" s="21"/>
+      <x:c r="W29"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="21"/>
@@ -1449,6 +1509,7 @@
       <x:c r="T30" s="21"/>
       <x:c r="U30" s="21"/>
       <x:c r="V30" s="21"/>
+      <x:c r="W30"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="21"/>
@@ -1473,6 +1534,7 @@
       <x:c r="T31" s="21"/>
       <x:c r="U31" s="21"/>
       <x:c r="V31" s="21"/>
+      <x:c r="W31"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="21"/>
@@ -1497,6 +1559,7 @@
       <x:c r="T32" s="21"/>
       <x:c r="U32" s="21"/>
       <x:c r="V32" s="21"/>
+      <x:c r="W32"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="21"/>
@@ -1521,6 +1584,7 @@
       <x:c r="T33" s="21"/>
       <x:c r="U33" s="21"/>
       <x:c r="V33" s="21"/>
+      <x:c r="W33"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="21"/>
@@ -1545,6 +1609,7 @@
       <x:c r="T34" s="21"/>
       <x:c r="U34" s="21"/>
       <x:c r="V34" s="21"/>
+      <x:c r="W34"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="21"/>
@@ -1569,6 +1634,7 @@
       <x:c r="T35" s="21"/>
       <x:c r="U35" s="21"/>
       <x:c r="V35" s="21"/>
+      <x:c r="W35"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="21"/>
@@ -1593,6 +1659,7 @@
       <x:c r="T36" s="21"/>
       <x:c r="U36" s="21"/>
       <x:c r="V36" s="21"/>
+      <x:c r="W36"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="21"/>
@@ -1617,6 +1684,7 @@
       <x:c r="T37" s="21"/>
       <x:c r="U37" s="21"/>
       <x:c r="V37" s="21"/>
+      <x:c r="W37"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="21"/>
@@ -1641,6 +1709,7 @@
       <x:c r="T38" s="21"/>
       <x:c r="U38" s="21"/>
       <x:c r="V38" s="21"/>
+      <x:c r="W38"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="21"/>
@@ -1665,6 +1734,7 @@
       <x:c r="T39" s="21"/>
       <x:c r="U39" s="21"/>
       <x:c r="V39" s="21"/>
+      <x:c r="W39"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="21"/>
@@ -1689,6 +1759,7 @@
       <x:c r="T40" s="21"/>
       <x:c r="U40" s="21"/>
       <x:c r="V40" s="21"/>
+      <x:c r="W40"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="21"/>
@@ -1713,6 +1784,7 @@
       <x:c r="T41" s="21"/>
       <x:c r="U41" s="21"/>
       <x:c r="V41" s="21"/>
+      <x:c r="W41"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="21"/>
@@ -1737,6 +1809,7 @@
       <x:c r="T42" s="21"/>
       <x:c r="U42" s="21"/>
       <x:c r="V42" s="21"/>
+      <x:c r="W42"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="21"/>
@@ -1761,6 +1834,7 @@
       <x:c r="T43" s="21"/>
       <x:c r="U43" s="21"/>
       <x:c r="V43" s="21"/>
+      <x:c r="W43"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="21"/>
@@ -1785,6 +1859,7 @@
       <x:c r="T44" s="21"/>
       <x:c r="U44" s="21"/>
       <x:c r="V44" s="21"/>
+      <x:c r="W44"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="21"/>
@@ -1809,6 +1884,7 @@
       <x:c r="T45" s="21"/>
       <x:c r="U45" s="21"/>
       <x:c r="V45" s="21"/>
+      <x:c r="W45"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="21"/>
@@ -1833,6 +1909,7 @@
       <x:c r="T46" s="21"/>
       <x:c r="U46" s="21"/>
       <x:c r="V46" s="21"/>
+      <x:c r="W46"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="21"/>
@@ -1857,6 +1934,7 @@
       <x:c r="T47" s="21"/>
       <x:c r="U47" s="21"/>
       <x:c r="V47" s="21"/>
+      <x:c r="W47"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="21"/>
@@ -1881,6 +1959,7 @@
       <x:c r="T48" s="21"/>
       <x:c r="U48" s="21"/>
       <x:c r="V48" s="21"/>
+      <x:c r="W48"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="21"/>
@@ -1905,6 +1984,7 @@
       <x:c r="T49" s="21"/>
       <x:c r="U49" s="21"/>
       <x:c r="V49" s="21"/>
+      <x:c r="W49"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="21"/>
@@ -1929,6 +2009,7 @@
       <x:c r="T50" s="21"/>
       <x:c r="U50" s="21"/>
       <x:c r="V50" s="21"/>
+      <x:c r="W50"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="21"/>
@@ -1953,6 +2034,7 @@
       <x:c r="T51" s="21"/>
       <x:c r="U51" s="21"/>
       <x:c r="V51" s="21"/>
+      <x:c r="W51"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="21"/>
@@ -1977,6 +2059,7 @@
       <x:c r="T52" s="21"/>
       <x:c r="U52" s="21"/>
       <x:c r="V52" s="21"/>
+      <x:c r="W52"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="21"/>
@@ -2001,6 +2084,7 @@
       <x:c r="T53" s="21"/>
       <x:c r="U53" s="21"/>
       <x:c r="V53" s="21"/>
+      <x:c r="W53"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="21"/>
@@ -2025,6 +2109,7 @@
       <x:c r="T54" s="21"/>
       <x:c r="U54" s="21"/>
       <x:c r="V54" s="21"/>
+      <x:c r="W54"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="21"/>
@@ -2049,6 +2134,7 @@
       <x:c r="T55" s="21"/>
       <x:c r="U55" s="21"/>
       <x:c r="V55" s="21"/>
+      <x:c r="W55"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="21"/>
@@ -2073,6 +2159,7 @@
       <x:c r="T56" s="21"/>
       <x:c r="U56" s="21"/>
       <x:c r="V56" s="21"/>
+      <x:c r="W56"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="21"/>
@@ -2097,6 +2184,7 @@
       <x:c r="T57" s="21"/>
       <x:c r="U57" s="21"/>
       <x:c r="V57" s="21"/>
+      <x:c r="W57"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="21"/>
@@ -2121,6 +2209,7 @@
       <x:c r="T58" s="21"/>
       <x:c r="U58" s="21"/>
       <x:c r="V58" s="21"/>
+      <x:c r="W58"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="21"/>
@@ -2145,6 +2234,7 @@
       <x:c r="T59" s="21"/>
       <x:c r="U59" s="21"/>
       <x:c r="V59" s="21"/>
+      <x:c r="W59"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="21"/>
@@ -2169,6 +2259,7 @@
       <x:c r="T60" s="21"/>
       <x:c r="U60" s="21"/>
       <x:c r="V60" s="21"/>
+      <x:c r="W60"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="21"/>
@@ -2193,6 +2284,7 @@
       <x:c r="T61" s="21"/>
       <x:c r="U61" s="21"/>
       <x:c r="V61" s="21"/>
+      <x:c r="W61"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="21"/>
@@ -2217,6 +2309,7 @@
       <x:c r="T62" s="21"/>
       <x:c r="U62" s="21"/>
       <x:c r="V62" s="21"/>
+      <x:c r="W62"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="21"/>
@@ -2241,6 +2334,7 @@
       <x:c r="T63" s="21"/>
       <x:c r="U63" s="21"/>
       <x:c r="V63" s="21"/>
+      <x:c r="W63"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="21"/>
@@ -2265,6 +2359,7 @@
       <x:c r="T64" s="21"/>
       <x:c r="U64" s="21"/>
       <x:c r="V64" s="21"/>
+      <x:c r="W64"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="21"/>
@@ -2289,6 +2384,7 @@
       <x:c r="T65" s="21"/>
       <x:c r="U65" s="21"/>
       <x:c r="V65" s="21"/>
+      <x:c r="W65"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="21"/>
@@ -2313,6 +2409,7 @@
       <x:c r="T66" s="21"/>
       <x:c r="U66" s="21"/>
       <x:c r="V66" s="21"/>
+      <x:c r="W66"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="21"/>
@@ -2337,6 +2434,7 @@
       <x:c r="T67" s="21"/>
       <x:c r="U67" s="21"/>
       <x:c r="V67" s="21"/>
+      <x:c r="W67"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="21"/>
@@ -2361,6 +2459,7 @@
       <x:c r="T68" s="21"/>
       <x:c r="U68" s="21"/>
       <x:c r="V68" s="21"/>
+      <x:c r="W68"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="21"/>
@@ -2385,6 +2484,7 @@
       <x:c r="T69" s="21"/>
       <x:c r="U69" s="21"/>
       <x:c r="V69" s="21"/>
+      <x:c r="W69"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="21"/>
@@ -2409,6 +2509,7 @@
       <x:c r="T70" s="21"/>
       <x:c r="U70" s="21"/>
       <x:c r="V70" s="21"/>
+      <x:c r="W70"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="21"/>
@@ -2433,6 +2534,7 @@
       <x:c r="T71" s="21"/>
       <x:c r="U71" s="21"/>
       <x:c r="V71" s="21"/>
+      <x:c r="W71"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="21"/>
@@ -2457,6 +2559,7 @@
       <x:c r="T72" s="21"/>
       <x:c r="U72" s="21"/>
       <x:c r="V72" s="21"/>
+      <x:c r="W72"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="21"/>
@@ -2481,6 +2584,7 @@
       <x:c r="T73" s="21"/>
       <x:c r="U73" s="21"/>
       <x:c r="V73" s="21"/>
+      <x:c r="W73"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="21"/>
@@ -2505,6 +2609,7 @@
       <x:c r="T74" s="21"/>
       <x:c r="U74" s="21"/>
       <x:c r="V74" s="21"/>
+      <x:c r="W74"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="21"/>
@@ -2529,6 +2634,7 @@
       <x:c r="T75" s="21"/>
       <x:c r="U75" s="21"/>
       <x:c r="V75" s="21"/>
+      <x:c r="W75"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="21"/>
@@ -2553,6 +2659,7 @@
       <x:c r="T76" s="21"/>
       <x:c r="U76" s="21"/>
       <x:c r="V76" s="21"/>
+      <x:c r="W76"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="21"/>
@@ -2577,6 +2684,7 @@
       <x:c r="T77" s="21"/>
       <x:c r="U77" s="21"/>
       <x:c r="V77" s="21"/>
+      <x:c r="W77"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="21"/>
@@ -2601,6 +2709,7 @@
       <x:c r="T78" s="21"/>
       <x:c r="U78" s="21"/>
       <x:c r="V78" s="21"/>
+      <x:c r="W78"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="21"/>
@@ -2625,6 +2734,7 @@
       <x:c r="T79" s="21"/>
       <x:c r="U79" s="21"/>
       <x:c r="V79" s="21"/>
+      <x:c r="W79"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="21"/>
@@ -2649,6 +2759,7 @@
       <x:c r="T80" s="21"/>
       <x:c r="U80" s="21"/>
       <x:c r="V80" s="21"/>
+      <x:c r="W80"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="21"/>
@@ -2673,6 +2784,7 @@
       <x:c r="T81" s="21"/>
       <x:c r="U81" s="21"/>
       <x:c r="V81" s="21"/>
+      <x:c r="W81"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="21"/>
@@ -2697,6 +2809,7 @@
       <x:c r="T82" s="21"/>
       <x:c r="U82" s="21"/>
       <x:c r="V82" s="21"/>
+      <x:c r="W82"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="21"/>
@@ -2721,6 +2834,7 @@
       <x:c r="T83" s="21"/>
       <x:c r="U83" s="21"/>
       <x:c r="V83" s="21"/>
+      <x:c r="W83"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="21"/>
@@ -2745,6 +2859,7 @@
       <x:c r="T84" s="21"/>
       <x:c r="U84" s="21"/>
       <x:c r="V84" s="21"/>
+      <x:c r="W84"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="21"/>
@@ -2769,6 +2884,7 @@
       <x:c r="T85" s="21"/>
       <x:c r="U85" s="21"/>
       <x:c r="V85" s="21"/>
+      <x:c r="W85"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="21"/>
@@ -2793,6 +2909,7 @@
       <x:c r="T86" s="21"/>
       <x:c r="U86" s="21"/>
       <x:c r="V86" s="21"/>
+      <x:c r="W86"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="21"/>
@@ -2817,6 +2934,7 @@
       <x:c r="T87" s="21"/>
       <x:c r="U87" s="21"/>
       <x:c r="V87" s="21"/>
+      <x:c r="W87"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="21"/>
@@ -2841,6 +2959,7 @@
       <x:c r="T88" s="21"/>
       <x:c r="U88" s="21"/>
       <x:c r="V88" s="21"/>
+      <x:c r="W88"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="21"/>
@@ -2865,6 +2984,7 @@
       <x:c r="T89" s="21"/>
       <x:c r="U89" s="21"/>
       <x:c r="V89" s="21"/>
+      <x:c r="W89"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="21"/>
@@ -2889,6 +3009,7 @@
       <x:c r="T90" s="21"/>
       <x:c r="U90" s="21"/>
       <x:c r="V90" s="21"/>
+      <x:c r="W90"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="21"/>
@@ -2913,6 +3034,7 @@
       <x:c r="T91" s="21"/>
       <x:c r="U91" s="21"/>
       <x:c r="V91" s="21"/>
+      <x:c r="W91"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="21"/>
@@ -2937,6 +3059,7 @@
       <x:c r="T92" s="21"/>
       <x:c r="U92" s="21"/>
       <x:c r="V92" s="21"/>
+      <x:c r="W92"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="21"/>
@@ -2961,6 +3084,7 @@
       <x:c r="T93" s="21"/>
       <x:c r="U93" s="21"/>
       <x:c r="V93" s="21"/>
+      <x:c r="W93"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="21"/>
@@ -2985,6 +3109,7 @@
       <x:c r="T94" s="21"/>
       <x:c r="U94" s="21"/>
       <x:c r="V94" s="21"/>
+      <x:c r="W94"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="21"/>
@@ -3009,6 +3134,7 @@
       <x:c r="T95" s="21"/>
       <x:c r="U95" s="21"/>
       <x:c r="V95" s="21"/>
+      <x:c r="W95"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="21"/>
@@ -3033,6 +3159,7 @@
       <x:c r="T96" s="21"/>
       <x:c r="U96" s="21"/>
       <x:c r="V96" s="21"/>
+      <x:c r="W96"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="21"/>
@@ -3057,6 +3184,7 @@
       <x:c r="T97" s="21"/>
       <x:c r="U97" s="21"/>
       <x:c r="V97" s="21"/>
+      <x:c r="W97"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="21"/>
@@ -3081,6 +3209,7 @@
       <x:c r="T98" s="21"/>
       <x:c r="U98" s="21"/>
       <x:c r="V98" s="21"/>
+      <x:c r="W98"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="21"/>
@@ -3105,6 +3234,7 @@
       <x:c r="T99" s="21"/>
       <x:c r="U99" s="21"/>
       <x:c r="V99" s="21"/>
+      <x:c r="W99"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="21"/>
@@ -3129,6 +3259,7 @@
       <x:c r="T100" s="21"/>
       <x:c r="U100" s="21"/>
       <x:c r="V100" s="21"/>
+      <x:c r="W100"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="21"/>
@@ -3153,6 +3284,7 @@
       <x:c r="T101" s="21"/>
       <x:c r="U101" s="21"/>
       <x:c r="V101" s="21"/>
+      <x:c r="W101"/>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="21"/>
@@ -3177,6 +3309,7 @@
       <x:c r="T102" s="21"/>
       <x:c r="U102" s="21"/>
       <x:c r="V102" s="21"/>
+      <x:c r="W102"/>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="21"/>
@@ -3201,6 +3334,7 @@
       <x:c r="T103" s="21"/>
       <x:c r="U103" s="21"/>
       <x:c r="V103" s="21"/>
+      <x:c r="W103"/>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="21"/>
@@ -3225,6 +3359,7 @@
       <x:c r="T104" s="21"/>
       <x:c r="U104" s="21"/>
       <x:c r="V104" s="21"/>
+      <x:c r="W104"/>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="21"/>
@@ -3249,6 +3384,7 @@
       <x:c r="T105" s="21"/>
       <x:c r="U105" s="21"/>
       <x:c r="V105" s="21"/>
+      <x:c r="W105"/>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="21"/>
@@ -3273,6 +3409,7 @@
       <x:c r="T106" s="21"/>
       <x:c r="U106" s="21"/>
       <x:c r="V106" s="21"/>
+      <x:c r="W106"/>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="21"/>
@@ -3297,6 +3434,7 @@
       <x:c r="T107" s="21"/>
       <x:c r="U107" s="21"/>
       <x:c r="V107" s="21"/>
+      <x:c r="W107"/>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="21"/>
@@ -3321,6 +3459,7 @@
       <x:c r="T108" s="21"/>
       <x:c r="U108" s="21"/>
       <x:c r="V108" s="21"/>
+      <x:c r="W108"/>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="21"/>
@@ -3345,6 +3484,7 @@
       <x:c r="T109" s="21"/>
       <x:c r="U109" s="21"/>
       <x:c r="V109" s="21"/>
+      <x:c r="W109"/>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="21"/>
@@ -3369,6 +3509,7 @@
       <x:c r="T110" s="21"/>
       <x:c r="U110" s="21"/>
       <x:c r="V110" s="21"/>
+      <x:c r="W110"/>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="21"/>
@@ -3393,6 +3534,7 @@
       <x:c r="T111" s="21"/>
       <x:c r="U111" s="21"/>
       <x:c r="V111" s="21"/>
+      <x:c r="W111"/>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="21"/>
@@ -3417,6 +3559,7 @@
       <x:c r="T112" s="21"/>
       <x:c r="U112" s="21"/>
       <x:c r="V112" s="21"/>
+      <x:c r="W112"/>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="21"/>
@@ -3441,6 +3584,7 @@
       <x:c r="T113" s="21"/>
       <x:c r="U113" s="21"/>
       <x:c r="V113" s="21"/>
+      <x:c r="W113"/>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="21"/>
@@ -3465,6 +3609,7 @@
       <x:c r="T114" s="21"/>
       <x:c r="U114" s="21"/>
       <x:c r="V114" s="21"/>
+      <x:c r="W114"/>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="21"/>
@@ -3489,6 +3634,7 @@
       <x:c r="T115" s="21"/>
       <x:c r="U115" s="21"/>
       <x:c r="V115" s="21"/>
+      <x:c r="W115"/>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="21"/>
@@ -3513,6 +3659,7 @@
       <x:c r="T116" s="21"/>
       <x:c r="U116" s="21"/>
       <x:c r="V116" s="21"/>
+      <x:c r="W116"/>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="21"/>
@@ -3537,6 +3684,7 @@
       <x:c r="T117" s="21"/>
       <x:c r="U117" s="21"/>
       <x:c r="V117" s="21"/>
+      <x:c r="W117"/>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="21"/>
@@ -3561,6 +3709,7 @@
       <x:c r="T118" s="21"/>
       <x:c r="U118" s="21"/>
       <x:c r="V118" s="21"/>
+      <x:c r="W118"/>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="21"/>
@@ -3585,6 +3734,7 @@
       <x:c r="T119" s="21"/>
       <x:c r="U119" s="21"/>
       <x:c r="V119" s="21"/>
+      <x:c r="W119"/>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="21"/>
@@ -3609,6 +3759,7 @@
       <x:c r="T120" s="21"/>
       <x:c r="U120" s="21"/>
       <x:c r="V120" s="21"/>
+      <x:c r="W120"/>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="21"/>
@@ -3633,6 +3784,7 @@
       <x:c r="T121" s="21"/>
       <x:c r="U121" s="21"/>
       <x:c r="V121" s="21"/>
+      <x:c r="W121"/>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="21"/>
@@ -3657,6 +3809,7 @@
       <x:c r="T122" s="21"/>
       <x:c r="U122" s="21"/>
       <x:c r="V122" s="21"/>
+      <x:c r="W122"/>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="21"/>
@@ -3681,6 +3834,7 @@
       <x:c r="T123" s="21"/>
       <x:c r="U123" s="21"/>
       <x:c r="V123" s="21"/>
+      <x:c r="W123"/>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="21"/>
@@ -3705,6 +3859,7 @@
       <x:c r="T124" s="21"/>
       <x:c r="U124" s="21"/>
       <x:c r="V124" s="21"/>
+      <x:c r="W124"/>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="21"/>
@@ -3729,6 +3884,7 @@
       <x:c r="T125" s="21"/>
       <x:c r="U125" s="21"/>
       <x:c r="V125" s="21"/>
+      <x:c r="W125"/>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="21"/>
@@ -3753,6 +3909,7 @@
       <x:c r="T126" s="21"/>
       <x:c r="U126" s="21"/>
       <x:c r="V126" s="21"/>
+      <x:c r="W126"/>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="21"/>
@@ -3777,6 +3934,7 @@
       <x:c r="T127" s="21"/>
       <x:c r="U127" s="21"/>
       <x:c r="V127" s="21"/>
+      <x:c r="W127"/>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="21"/>
@@ -3801,6 +3959,7 @@
       <x:c r="T128" s="21"/>
       <x:c r="U128" s="21"/>
       <x:c r="V128" s="21"/>
+      <x:c r="W128"/>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="21"/>
@@ -3825,6 +3984,7 @@
       <x:c r="T129" s="21"/>
       <x:c r="U129" s="21"/>
       <x:c r="V129" s="21"/>
+      <x:c r="W129"/>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="21"/>
@@ -3849,6 +4009,7 @@
       <x:c r="T130" s="21"/>
       <x:c r="U130" s="21"/>
       <x:c r="V130" s="21"/>
+      <x:c r="W130"/>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="21"/>
@@ -3873,6 +4034,7 @@
       <x:c r="T131" s="21"/>
       <x:c r="U131" s="21"/>
       <x:c r="V131" s="21"/>
+      <x:c r="W131"/>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="21"/>
@@ -3897,6 +4059,7 @@
       <x:c r="T132" s="21"/>
       <x:c r="U132" s="21"/>
       <x:c r="V132" s="21"/>
+      <x:c r="W132"/>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="21"/>
@@ -3921,6 +4084,7 @@
       <x:c r="T133" s="21"/>
       <x:c r="U133" s="21"/>
       <x:c r="V133" s="21"/>
+      <x:c r="W133"/>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="21"/>
@@ -3945,6 +4109,7 @@
       <x:c r="T134" s="21"/>
       <x:c r="U134" s="21"/>
       <x:c r="V134" s="21"/>
+      <x:c r="W134"/>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="21"/>
@@ -3969,6 +4134,7 @@
       <x:c r="T135" s="21"/>
       <x:c r="U135" s="21"/>
       <x:c r="V135" s="21"/>
+      <x:c r="W135"/>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="21"/>
@@ -3993,6 +4159,7 @@
       <x:c r="T136" s="21"/>
       <x:c r="U136" s="21"/>
       <x:c r="V136" s="21"/>
+      <x:c r="W136"/>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="21"/>
@@ -4017,6 +4184,7 @@
       <x:c r="T137" s="21"/>
       <x:c r="U137" s="21"/>
       <x:c r="V137" s="21"/>
+      <x:c r="W137"/>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="21"/>
@@ -4041,6 +4209,7 @@
       <x:c r="T138" s="21"/>
       <x:c r="U138" s="21"/>
       <x:c r="V138" s="21"/>
+      <x:c r="W138"/>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="21"/>
@@ -4065,6 +4234,7 @@
       <x:c r="T139" s="21"/>
       <x:c r="U139" s="21"/>
       <x:c r="V139" s="21"/>
+      <x:c r="W139"/>
     </x:row>
     <x:row r="140">
       <x:c r="A140" s="21"/>
@@ -4089,6 +4259,7 @@
       <x:c r="T140" s="21"/>
       <x:c r="U140" s="21"/>
       <x:c r="V140" s="21"/>
+      <x:c r="W140"/>
     </x:row>
     <x:row r="141">
       <x:c r="A141" s="21"/>
@@ -4113,6 +4284,7 @@
       <x:c r="T141" s="21"/>
       <x:c r="U141" s="21"/>
       <x:c r="V141" s="21"/>
+      <x:c r="W141"/>
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="21"/>
@@ -4137,6 +4309,7 @@
       <x:c r="T142" s="21"/>
       <x:c r="U142" s="21"/>
       <x:c r="V142" s="21"/>
+      <x:c r="W142"/>
     </x:row>
     <x:row r="143">
       <x:c r="A143" s="21"/>
@@ -4161,6 +4334,7 @@
       <x:c r="T143" s="21"/>
       <x:c r="U143" s="21"/>
       <x:c r="V143" s="21"/>
+      <x:c r="W143"/>
     </x:row>
     <x:row r="144">
       <x:c r="A144" s="21"/>
@@ -4185,6 +4359,7 @@
       <x:c r="T144" s="21"/>
       <x:c r="U144" s="21"/>
       <x:c r="V144" s="21"/>
+      <x:c r="W144"/>
     </x:row>
     <x:row r="145">
       <x:c r="A145" s="21"/>
@@ -4209,6 +4384,7 @@
       <x:c r="T145" s="21"/>
       <x:c r="U145" s="21"/>
       <x:c r="V145" s="21"/>
+      <x:c r="W145"/>
     </x:row>
     <x:row r="146">
       <x:c r="A146" s="21"/>
@@ -4233,6 +4409,7 @@
       <x:c r="T146" s="21"/>
       <x:c r="U146" s="21"/>
       <x:c r="V146" s="21"/>
+      <x:c r="W146"/>
     </x:row>
     <x:row r="147">
       <x:c r="A147" s="21"/>
@@ -4257,6 +4434,7 @@
       <x:c r="T147" s="21"/>
       <x:c r="U147" s="21"/>
       <x:c r="V147" s="21"/>
+      <x:c r="W147"/>
     </x:row>
     <x:row r="148">
       <x:c r="A148" s="21"/>
@@ -4281,6 +4459,7 @@
       <x:c r="T148" s="21"/>
       <x:c r="U148" s="21"/>
       <x:c r="V148" s="21"/>
+      <x:c r="W148"/>
     </x:row>
     <x:row r="149">
       <x:c r="A149" s="21"/>
@@ -4305,6 +4484,7 @@
       <x:c r="T149" s="21"/>
       <x:c r="U149" s="21"/>
       <x:c r="V149" s="21"/>
+      <x:c r="W149"/>
     </x:row>
     <x:row r="150">
       <x:c r="A150" s="21"/>
@@ -4329,6 +4509,7 @@
       <x:c r="T150" s="21"/>
       <x:c r="U150" s="21"/>
       <x:c r="V150" s="21"/>
+      <x:c r="W150"/>
     </x:row>
     <x:row r="151">
       <x:c r="A151" s="21"/>
@@ -4353,6 +4534,7 @@
       <x:c r="T151" s="21"/>
       <x:c r="U151" s="21"/>
       <x:c r="V151" s="21"/>
+      <x:c r="W151"/>
     </x:row>
     <x:row r="152">
       <x:c r="A152" s="21"/>
@@ -4377,6 +4559,7 @@
       <x:c r="T152" s="21"/>
       <x:c r="U152" s="21"/>
       <x:c r="V152" s="21"/>
+      <x:c r="W152"/>
     </x:row>
     <x:row r="153">
       <x:c r="A153" s="21"/>
@@ -4401,6 +4584,7 @@
       <x:c r="T153" s="21"/>
       <x:c r="U153" s="21"/>
       <x:c r="V153" s="21"/>
+      <x:c r="W153"/>
     </x:row>
     <x:row r="154">
       <x:c r="A154" s="21"/>
@@ -4425,6 +4609,7 @@
       <x:c r="T154" s="21"/>
       <x:c r="U154" s="21"/>
       <x:c r="V154" s="21"/>
+      <x:c r="W154"/>
     </x:row>
     <x:row r="155">
       <x:c r="A155" s="21"/>
@@ -4449,6 +4634,7 @@
       <x:c r="T155" s="21"/>
       <x:c r="U155" s="21"/>
       <x:c r="V155" s="21"/>
+      <x:c r="W155"/>
     </x:row>
     <x:row r="156">
       <x:c r="A156" s="21"/>
@@ -4473,6 +4659,7 @@
       <x:c r="T156" s="21"/>
       <x:c r="U156" s="21"/>
       <x:c r="V156" s="21"/>
+      <x:c r="W156"/>
     </x:row>
     <x:row r="157">
       <x:c r="A157" s="21"/>
@@ -4497,6 +4684,7 @@
       <x:c r="T157" s="21"/>
       <x:c r="U157" s="21"/>
       <x:c r="V157" s="21"/>
+      <x:c r="W157"/>
     </x:row>
     <x:row r="158">
       <x:c r="A158" s="21"/>
@@ -4521,6 +4709,7 @@
       <x:c r="T158" s="21"/>
       <x:c r="U158" s="21"/>
       <x:c r="V158" s="21"/>
+      <x:c r="W158"/>
     </x:row>
     <x:row r="159">
       <x:c r="A159" s="21"/>
@@ -4545,6 +4734,7 @@
       <x:c r="T159" s="21"/>
       <x:c r="U159" s="21"/>
       <x:c r="V159" s="21"/>
+      <x:c r="W159"/>
     </x:row>
     <x:row r="160">
       <x:c r="A160" s="21"/>
@@ -4569,6 +4759,7 @@
       <x:c r="T160" s="21"/>
       <x:c r="U160" s="21"/>
       <x:c r="V160" s="21"/>
+      <x:c r="W160"/>
     </x:row>
     <x:row r="161">
       <x:c r="A161" s="21"/>
@@ -4593,6 +4784,7 @@
       <x:c r="T161" s="21"/>
       <x:c r="U161" s="21"/>
       <x:c r="V161" s="21"/>
+      <x:c r="W161"/>
     </x:row>
     <x:row r="162">
       <x:c r="A162" s="21"/>
@@ -4617,6 +4809,7 @@
       <x:c r="T162" s="21"/>
       <x:c r="U162" s="21"/>
       <x:c r="V162" s="21"/>
+      <x:c r="W162"/>
     </x:row>
     <x:row r="163">
       <x:c r="A163" s="21"/>
@@ -4641,6 +4834,7 @@
       <x:c r="T163" s="21"/>
       <x:c r="U163" s="21"/>
       <x:c r="V163" s="21"/>
+      <x:c r="W163"/>
     </x:row>
     <x:row r="164">
       <x:c r="A164" s="21"/>
@@ -4665,6 +4859,7 @@
       <x:c r="T164" s="21"/>
       <x:c r="U164" s="21"/>
       <x:c r="V164" s="21"/>
+      <x:c r="W164"/>
     </x:row>
     <x:row r="165">
       <x:c r="A165" s="21"/>
@@ -4689,6 +4884,7 @@
       <x:c r="T165" s="21"/>
       <x:c r="U165" s="21"/>
       <x:c r="V165" s="21"/>
+      <x:c r="W165"/>
     </x:row>
     <x:row r="166">
       <x:c r="A166" s="21"/>
@@ -4713,6 +4909,7 @@
       <x:c r="T166" s="21"/>
       <x:c r="U166" s="21"/>
       <x:c r="V166" s="21"/>
+      <x:c r="W166"/>
     </x:row>
     <x:row r="167">
       <x:c r="A167" s="21"/>
@@ -4737,6 +4934,7 @@
       <x:c r="T167" s="21"/>
       <x:c r="U167" s="21"/>
       <x:c r="V167" s="21"/>
+      <x:c r="W167"/>
     </x:row>
     <x:row r="168">
       <x:c r="A168" s="21"/>
@@ -4761,6 +4959,7 @@
       <x:c r="T168" s="21"/>
       <x:c r="U168" s="21"/>
       <x:c r="V168" s="21"/>
+      <x:c r="W168"/>
     </x:row>
     <x:row r="169">
       <x:c r="A169" s="21"/>
@@ -4785,6 +4984,7 @@
       <x:c r="T169" s="21"/>
       <x:c r="U169" s="21"/>
       <x:c r="V169" s="21"/>
+      <x:c r="W169"/>
     </x:row>
     <x:row r="170">
       <x:c r="A170" s="21"/>
@@ -4809,6 +5009,7 @@
       <x:c r="T170" s="21"/>
       <x:c r="U170" s="21"/>
       <x:c r="V170" s="21"/>
+      <x:c r="W170"/>
     </x:row>
     <x:row r="171">
       <x:c r="A171" s="21"/>
@@ -4833,6 +5034,7 @@
       <x:c r="T171" s="21"/>
       <x:c r="U171" s="21"/>
       <x:c r="V171" s="21"/>
+      <x:c r="W171"/>
     </x:row>
     <x:row r="172">
       <x:c r="A172" s="21"/>
@@ -4857,6 +5059,7 @@
       <x:c r="T172" s="21"/>
       <x:c r="U172" s="21"/>
       <x:c r="V172" s="21"/>
+      <x:c r="W172"/>
     </x:row>
     <x:row r="173">
       <x:c r="A173" s="21"/>
@@ -4881,6 +5084,7 @@
       <x:c r="T173" s="21"/>
       <x:c r="U173" s="21"/>
       <x:c r="V173" s="21"/>
+      <x:c r="W173"/>
     </x:row>
     <x:row r="174">
       <x:c r="A174" s="21"/>
@@ -4905,6 +5109,7 @@
       <x:c r="T174" s="21"/>
       <x:c r="U174" s="21"/>
       <x:c r="V174" s="21"/>
+      <x:c r="W174"/>
     </x:row>
     <x:row r="175">
       <x:c r="A175" s="21"/>
@@ -4929,6 +5134,7 @@
       <x:c r="T175" s="21"/>
       <x:c r="U175" s="21"/>
       <x:c r="V175" s="21"/>
+      <x:c r="W175"/>
     </x:row>
     <x:row r="176">
       <x:c r="A176" s="21"/>
@@ -4953,6 +5159,7 @@
       <x:c r="T176" s="21"/>
       <x:c r="U176" s="21"/>
       <x:c r="V176" s="21"/>
+      <x:c r="W176"/>
     </x:row>
     <x:row r="177">
       <x:c r="A177" s="21"/>
@@ -4977,6 +5184,7 @@
       <x:c r="T177" s="21"/>
       <x:c r="U177" s="21"/>
       <x:c r="V177" s="21"/>
+      <x:c r="W177"/>
     </x:row>
     <x:row r="178">
       <x:c r="A178" s="21"/>
@@ -5001,6 +5209,7 @@
       <x:c r="T178" s="21"/>
       <x:c r="U178" s="21"/>
       <x:c r="V178" s="21"/>
+      <x:c r="W178"/>
     </x:row>
     <x:row r="179">
       <x:c r="A179" s="21"/>
@@ -5025,6 +5234,7 @@
       <x:c r="T179" s="21"/>
       <x:c r="U179" s="21"/>
       <x:c r="V179" s="21"/>
+      <x:c r="W179"/>
     </x:row>
     <x:row r="180">
       <x:c r="A180" s="21"/>
@@ -5049,6 +5259,7 @@
       <x:c r="T180" s="21"/>
       <x:c r="U180" s="21"/>
       <x:c r="V180" s="21"/>
+      <x:c r="W180"/>
     </x:row>
     <x:row r="181">
       <x:c r="A181" s="21"/>
@@ -5073,6 +5284,7 @@
       <x:c r="T181" s="21"/>
       <x:c r="U181" s="21"/>
       <x:c r="V181" s="21"/>
+      <x:c r="W181"/>
     </x:row>
     <x:row r="182">
       <x:c r="A182" s="21"/>
@@ -5097,6 +5309,7 @@
       <x:c r="T182" s="21"/>
       <x:c r="U182" s="21"/>
       <x:c r="V182" s="21"/>
+      <x:c r="W182"/>
     </x:row>
     <x:row r="183">
       <x:c r="A183" s="21"/>
@@ -5121,6 +5334,7 @@
       <x:c r="T183" s="21"/>
       <x:c r="U183" s="21"/>
       <x:c r="V183" s="21"/>
+      <x:c r="W183"/>
     </x:row>
     <x:row r="184">
       <x:c r="A184" s="21"/>
@@ -5145,6 +5359,7 @@
       <x:c r="T184" s="21"/>
       <x:c r="U184" s="21"/>
       <x:c r="V184" s="21"/>
+      <x:c r="W184"/>
     </x:row>
     <x:row r="185">
       <x:c r="A185" s="21"/>
@@ -5169,6 +5384,7 @@
       <x:c r="T185" s="21"/>
       <x:c r="U185" s="21"/>
       <x:c r="V185" s="21"/>
+      <x:c r="W185"/>
     </x:row>
     <x:row r="186">
       <x:c r="A186" s="21"/>
@@ -5193,6 +5409,7 @@
       <x:c r="T186" s="21"/>
       <x:c r="U186" s="21"/>
       <x:c r="V186" s="21"/>
+      <x:c r="W186"/>
     </x:row>
     <x:row r="187">
       <x:c r="A187" s="21"/>
@@ -5217,6 +5434,7 @@
       <x:c r="T187" s="21"/>
       <x:c r="U187" s="21"/>
       <x:c r="V187" s="21"/>
+      <x:c r="W187"/>
     </x:row>
     <x:row r="188">
       <x:c r="A188" s="21"/>
@@ -5241,6 +5459,7 @@
       <x:c r="T188" s="21"/>
       <x:c r="U188" s="21"/>
       <x:c r="V188" s="21"/>
+      <x:c r="W188"/>
     </x:row>
     <x:row r="189">
       <x:c r="A189" s="21"/>
@@ -5265,6 +5484,7 @@
       <x:c r="T189" s="21"/>
       <x:c r="U189" s="21"/>
       <x:c r="V189" s="21"/>
+      <x:c r="W189"/>
     </x:row>
     <x:row r="190">
       <x:c r="A190" s="21"/>
@@ -5289,6 +5509,7 @@
       <x:c r="T190" s="21"/>
       <x:c r="U190" s="21"/>
       <x:c r="V190" s="21"/>
+      <x:c r="W190"/>
     </x:row>
     <x:row r="191">
       <x:c r="A191" s="21"/>
@@ -5313,6 +5534,7 @@
       <x:c r="T191" s="21"/>
       <x:c r="U191" s="21"/>
       <x:c r="V191" s="21"/>
+      <x:c r="W191"/>
     </x:row>
     <x:row r="192">
       <x:c r="A192" s="21"/>
@@ -5337,6 +5559,7 @@
       <x:c r="T192" s="21"/>
       <x:c r="U192" s="21"/>
       <x:c r="V192" s="21"/>
+      <x:c r="W192"/>
     </x:row>
     <x:row r="193">
       <x:c r="A193" s="21"/>
@@ -5361,6 +5584,7 @@
       <x:c r="T193" s="21"/>
       <x:c r="U193" s="21"/>
       <x:c r="V193" s="21"/>
+      <x:c r="W193"/>
     </x:row>
     <x:row r="194">
       <x:c r="A194" s="21"/>
@@ -5385,6 +5609,7 @@
       <x:c r="T194" s="21"/>
       <x:c r="U194" s="21"/>
       <x:c r="V194" s="21"/>
+      <x:c r="W194"/>
     </x:row>
     <x:row r="195">
       <x:c r="A195" s="21"/>
@@ -5409,6 +5634,7 @@
       <x:c r="T195" s="21"/>
       <x:c r="U195" s="21"/>
       <x:c r="V195" s="21"/>
+      <x:c r="W195"/>
     </x:row>
     <x:row r="196">
       <x:c r="A196" s="21"/>
@@ -5433,6 +5659,7 @@
       <x:c r="T196" s="21"/>
       <x:c r="U196" s="21"/>
       <x:c r="V196" s="21"/>
+      <x:c r="W196"/>
     </x:row>
     <x:row r="197">
       <x:c r="A197" s="21"/>
@@ -5457,6 +5684,7 @@
       <x:c r="T197" s="21"/>
       <x:c r="U197" s="21"/>
       <x:c r="V197" s="21"/>
+      <x:c r="W197"/>
     </x:row>
     <x:row r="198">
       <x:c r="A198" s="21"/>
@@ -5481,6 +5709,7 @@
       <x:c r="T198" s="21"/>
       <x:c r="U198" s="21"/>
       <x:c r="V198" s="21"/>
+      <x:c r="W198"/>
     </x:row>
     <x:row r="199">
       <x:c r="A199" s="21"/>
@@ -5505,6 +5734,7 @@
       <x:c r="T199" s="21"/>
       <x:c r="U199" s="21"/>
       <x:c r="V199" s="21"/>
+      <x:c r="W199"/>
     </x:row>
     <x:row r="200">
       <x:c r="A200" s="21"/>
@@ -5529,6 +5759,7 @@
       <x:c r="T200" s="21"/>
       <x:c r="U200" s="21"/>
       <x:c r="V200" s="21"/>
+      <x:c r="W200"/>
     </x:row>
     <x:row r="201">
       <x:c r="A201" s="21"/>
@@ -12735,7 +12966,7 @@
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="异常"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="异常"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="4">
+  <x:dataValidations count="8">
     <x:dataValidation type="list" sqref="B2:B500">
       <x:formula1>"MX,US"</x:formula1>
     </x:dataValidation>
@@ -12746,6 +12977,18 @@
       <x:formula1>"新刚,志恒,康德,宇航,熊,德,恒"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="U2:U500">
+      <x:formula1>"正常,待复核（源表错列）"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="B2:B200">
+      <x:formula1>"MX,US"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I2:I200">
+      <x:formula1>"未绑定,已绑定,已登录,异常,封号,停用"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="M2:M200">
+      <x:formula1>"新刚,志恒,康德,宇航,熊,德,恒"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="V2:V200">
       <x:formula1>"正常,待复核（源表错列）"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -12787,7 +13030,7 @@
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="98" t="str">
-        <x:v>前14列保持小犀代采 API 与 TSV 契约；后8列镜像现有飞书运营字段。Excel 导入后仍需在飞书中手动设置系统字段、字段样式和单选项。</x:v>
+        <x:v>自「站点」至「绑定时间」连续13列保持小犀代采 API 写回与 TSV 契约；第1列「账号ID」和末尾9列为飞书系统/运营字段，其中「首次登录日期」仍纳入只读字段预检但当前建环境 API 不写入。Excel 导入后仍需手动设置字段样式和单选项。</x:v>
       </x:c>
       <x:c r="B2" s="98" t="str">
         <x:v>前14列保持小犀代采 API 与 TSV 契约；后8列镜像现有飞书运营字段。Excel 导入后仍需在飞书中手动设置系统字段、字段样式和单选项。</x:v>
@@ -13027,87 +13270,87 @@
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
       <x:c r="A15" s="50" t="str">
-        <x:v>环境序号</x:v>
+        <x:v>环境分组名</x:v>
       </x:c>
       <x:c r="B15" s="48" t="str">
-        <x:v>数字</x:v>
+        <x:v>文本</x:v>
       </x:c>
       <x:c r="C15" s="48" t="str">
-        <x:v>整数</x:v>
+        <x:v>plain</x:v>
       </x:c>
       <x:c r="D15" s="48" t="str">
-        <x:v>绑定写回</x:v>
+        <x:v>环境分组回写</x:v>
       </x:c>
       <x:c r="E15" s="108" t="str">
         <x:v>API 必需</x:v>
       </x:c>
       <x:c r="F15" s="48" t="str">
-        <x:v>对应 HubStudio serialNumber</x:v>
+        <x:v>记录 HubStudio 当前分组；环境移动分组时更新原记录，不新增重复买家号</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
       <x:c r="A16" s="50" t="str">
-        <x:v>采购员</x:v>
+        <x:v>环境序号</x:v>
       </x:c>
       <x:c r="B16" s="48" t="str">
-        <x:v>单选</x:v>
+        <x:v>数字</x:v>
       </x:c>
       <x:c r="C16" s="48" t="str">
-        <x:v>新刚、志恒、康德、宇航、熊、德、恒</x:v>
+        <x:v>整数</x:v>
       </x:c>
       <x:c r="D16" s="48" t="str">
-        <x:v>归属写回</x:v>
+        <x:v>绑定写回</x:v>
       </x:c>
       <x:c r="E16" s="108" t="str">
         <x:v>API 必需</x:v>
       </x:c>
       <x:c r="F16" s="48" t="str">
-        <x:v>前4项为当前系统名单，后3项兼容历史记录</x:v>
+        <x:v>对应 HubStudio serialNumber</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
       <x:c r="A17" s="50" t="str">
-        <x:v>绑定时间</x:v>
+        <x:v>采购员</x:v>
       </x:c>
       <x:c r="B17" s="48" t="str">
-        <x:v>日期</x:v>
+        <x:v>单选</x:v>
       </x:c>
       <x:c r="C17" s="48" t="str">
-        <x:v>yyyy-mm-dd hh:mm</x:v>
+        <x:v>新刚、志恒、康德、宇航、熊、德、恒</x:v>
       </x:c>
       <x:c r="D17" s="48" t="str">
-        <x:v>绑定写回</x:v>
+        <x:v>归属写回</x:v>
       </x:c>
       <x:c r="E17" s="108" t="str">
         <x:v>API 必需</x:v>
       </x:c>
       <x:c r="F17" s="48" t="str">
-        <x:v>使用北京时间，与现有表显示到分钟一致</x:v>
+        <x:v>前4项为当前系统名单，后3项兼容历史记录</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
       <x:c r="A18" s="50" t="str">
-        <x:v>首次登录日期</x:v>
+        <x:v>绑定时间</x:v>
       </x:c>
       <x:c r="B18" s="48" t="str">
         <x:v>日期</x:v>
       </x:c>
       <x:c r="C18" s="48" t="str">
-        <x:v>yyyy-mm-dd</x:v>
+        <x:v>yyyy-mm-dd hh:mm</x:v>
       </x:c>
       <x:c r="D18" s="48" t="str">
-        <x:v>注册/登录回写</x:v>
+        <x:v>绑定写回</x:v>
       </x:c>
       <x:c r="E18" s="108" t="str">
         <x:v>API 必需</x:v>
       </x:c>
       <x:c r="F18" s="48" t="str">
-        <x:v>与现有表日期显示一致</x:v>
+        <x:v>使用北京时间，与现有表显示到分钟一致</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="30" customHeight="1">
       <x:c r="A19" s="50" t="str">
-        <x:v>最后使用日期</x:v>
+        <x:v>首次登录日期</x:v>
       </x:c>
       <x:c r="B19" s="48" t="str">
         <x:v>日期</x:v>
@@ -13116,67 +13359,67 @@
         <x:v>yyyy-mm-dd</x:v>
       </x:c>
       <x:c r="D19" s="48" t="str">
-        <x:v>运营维护</x:v>
+        <x:v>登录历史</x:v>
       </x:c>
       <x:c r="E19" s="111" t="str">
-        <x:v>现有表镜像</x:v>
+        <x:v>字段预检必需</x:v>
       </x:c>
       <x:c r="F19" s="48" t="str">
-        <x:v>API 当前不写入</x:v>
+        <x:v>与现有表日期显示一致；当前买家号建环境 API 不写入</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="30" customHeight="1">
       <x:c r="A20" s="50" t="str">
-        <x:v>创建时间</x:v>
+        <x:v>最后使用日期</x:v>
       </x:c>
       <x:c r="B20" s="48" t="str">
-        <x:v>创建时间</x:v>
+        <x:v>日期</x:v>
       </x:c>
       <x:c r="C20" s="48" t="str">
         <x:v>yyyy-mm-dd</x:v>
       </x:c>
       <x:c r="D20" s="48" t="str">
-        <x:v>飞书系统审计</x:v>
+        <x:v>运营维护</x:v>
       </x:c>
       <x:c r="E20" s="111" t="str">
         <x:v>现有表镜像</x:v>
       </x:c>
       <x:c r="F20" s="48" t="str">
-        <x:v>导入后手动新增飞书系统字段</x:v>
+        <x:v>API 当前不写入</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="30" customHeight="1">
       <x:c r="A21" s="50" t="str">
-        <x:v>备注</x:v>
+        <x:v>创建时间</x:v>
       </x:c>
       <x:c r="B21" s="48" t="str">
-        <x:v>文本</x:v>
+        <x:v>创建时间</x:v>
       </x:c>
       <x:c r="C21" s="48" t="str">
-        <x:v>plain</x:v>
+        <x:v>yyyy-mm-dd</x:v>
       </x:c>
       <x:c r="D21" s="48" t="str">
-        <x:v>运营备注</x:v>
+        <x:v>飞书系统审计</x:v>
       </x:c>
       <x:c r="E21" s="111" t="str">
         <x:v>现有表镜像</x:v>
       </x:c>
       <x:c r="F21" s="48" t="str">
-        <x:v>API 当前不写入</x:v>
+        <x:v>导入后手动新增飞书系统字段</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="30" customHeight="1">
       <x:c r="A22" s="50" t="str">
-        <x:v>累计下单数</x:v>
+        <x:v>备注</x:v>
       </x:c>
       <x:c r="B22" s="48" t="str">
-        <x:v>数字</x:v>
+        <x:v>文本</x:v>
       </x:c>
       <x:c r="C22" s="48" t="str">
-        <x:v>整数</x:v>
+        <x:v>plain</x:v>
       </x:c>
       <x:c r="D22" s="48" t="str">
-        <x:v>运营统计</x:v>
+        <x:v>运营备注</x:v>
       </x:c>
       <x:c r="E22" s="111" t="str">
         <x:v>现有表镜像</x:v>
@@ -13187,16 +13430,16 @@
     </x:row>
     <x:row r="23" ht="30" customHeight="1">
       <x:c r="A23" s="50" t="str">
-        <x:v>异常记录</x:v>
+        <x:v>累计下单数</x:v>
       </x:c>
       <x:c r="B23" s="48" t="str">
-        <x:v>文本</x:v>
+        <x:v>数字</x:v>
       </x:c>
       <x:c r="C23" s="48" t="str">
-        <x:v>plain</x:v>
+        <x:v>整数</x:v>
       </x:c>
       <x:c r="D23" s="48" t="str">
-        <x:v>异常留痕</x:v>
+        <x:v>运营统计</x:v>
       </x:c>
       <x:c r="E23" s="111" t="str">
         <x:v>现有表镜像</x:v>
@@ -13207,61 +13450,81 @@
     </x:row>
     <x:row r="24" ht="30" customHeight="1">
       <x:c r="A24" s="50" t="str">
-        <x:v>创建人</x:v>
+        <x:v>异常记录</x:v>
       </x:c>
       <x:c r="B24" s="48" t="str">
-        <x:v>创建人</x:v>
+        <x:v>文本</x:v>
       </x:c>
       <x:c r="C24" s="48" t="str">
-        <x:v>飞书用户</x:v>
+        <x:v>plain</x:v>
       </x:c>
       <x:c r="D24" s="48" t="str">
-        <x:v>飞书系统审计</x:v>
+        <x:v>异常留痕</x:v>
       </x:c>
       <x:c r="E24" s="111" t="str">
         <x:v>现有表镜像</x:v>
       </x:c>
       <x:c r="F24" s="48" t="str">
-        <x:v>导入后手动新增飞书系统字段</x:v>
+        <x:v>API 当前不写入</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="30" customHeight="1">
       <x:c r="A25" s="50" t="str">
-        <x:v>迁移状态</x:v>
+        <x:v>创建人</x:v>
       </x:c>
       <x:c r="B25" s="48" t="str">
-        <x:v>单选</x:v>
+        <x:v>创建人</x:v>
       </x:c>
       <x:c r="C25" s="48" t="str">
-        <x:v>正常、待复核（源表错列）</x:v>
+        <x:v>飞书用户</x:v>
       </x:c>
       <x:c r="D25" s="48" t="str">
-        <x:v>历史迁移复核</x:v>
+        <x:v>飞书系统审计</x:v>
       </x:c>
       <x:c r="E25" s="111" t="str">
         <x:v>现有表镜像</x:v>
       </x:c>
       <x:c r="F25" s="48" t="str">
-        <x:v>选项与现有表完全一致</x:v>
+        <x:v>导入后手动新增飞书系统字段</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="30" customHeight="1">
       <x:c r="A26" s="50" t="str">
-        <x:v>操作人</x:v>
+        <x:v>迁移状态</x:v>
       </x:c>
       <x:c r="B26" s="48" t="str">
-        <x:v>人员</x:v>
+        <x:v>单选</x:v>
       </x:c>
       <x:c r="C26" s="48" t="str">
-        <x:v>飞书用户</x:v>
+        <x:v>正常、待复核（源表错列）</x:v>
       </x:c>
       <x:c r="D26" s="48" t="str">
-        <x:v>运营归属</x:v>
+        <x:v>历史迁移复核</x:v>
       </x:c>
       <x:c r="E26" s="111" t="str">
         <x:v>现有表镜像</x:v>
       </x:c>
       <x:c r="F26" s="48" t="str">
+        <x:v>选项与现有表完全一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>操作人</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>人员</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>飞书用户</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>运营归属</x:v>
+      </x:c>
+      <x:c r="E27" t="str">
+        <x:v>现有表镜像</x:v>
+      </x:c>
+      <x:c r="F27" t="str">
         <x:v>人员字段，API 当前不写入</x:v>
       </x:c>
     </x:row>
@@ -13302,7 +13565,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B30" s="119" t="str">
-        <x:v>保持前14列顺序；按字段说明设置类型、显示格式、文本样式和单选项。</x:v>
+        <x:v>保持从「站点」至「绑定时间」连续13列顺序；「首次登录日期」也需按字段说明创建并设置类型。</x:v>
       </x:c>
       <x:c r="C30" s="119"/>
       <x:c r="D30" s="119"/>

</xml_diff>